<commit_message>
DVS 2.0 v2: change request 06-10 (step log, checker revert, persona, audit)
Dropdown select/read by visible text, persona detection, Step_Log sheet and
log file, Checker revert recovery with Maker-Checker compare, tab-switch
persistence, Item Error List checks, record data audit, customer id lists in
config (dvs.cust.individual/minor/le), test data v2. Dry-run verified only;
not yet run against the live DVS app.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData/DVS/DVS_Automation_TestData.xlsx
+++ b/src/test/resources/TestData/DVS/DVS_Automation_TestData.xlsx
@@ -17,6 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DOCUMENT_MAPPING" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IMAGE_MAPPING" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REGRESSION" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="STEP_LOG_TEMPLATE" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'IMAGE_NAME_RULES'!$A$1:$F$9</definedName>
@@ -28,6 +29,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'DOCUMENT_MAPPING'!$A$1:$AC$128</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'IMAGE_MAPPING'!$A$1:$AC$66</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'REGRESSION'!$A$1:$AC$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'STEP_LOG_TEMPLATE'!$A$1:$V$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -486,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -664,66 +666,117 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>run.mode</t>
+          <t>keep.bug.value</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>COMBINED</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>POSITIVE_ONLY / NEGATIVE_ONLY / COMBINED / REGRESSION</t>
+          <t>After checker revert keep the accepted bug value and continue</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>restore.mode</t>
+          <t>data.audit</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>GROUP_END</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>GROUP_END = apply last positive data after each connected group; ROW = after every row</t>
+          <t>Pre-scan every record before scenarios</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>checker.flow</t>
+          <t>tabswitch.check</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>LATER</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>admin login only for now</t>
+          <t>Verify value after tab switch and reload</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>run.mode</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>COMBINED</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>POSITIVE_ONLY / NEGATIVE_ONLY / COMBINED / REGRESSION</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>restore.mode</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>GROUP_END</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>GROUP_END = apply last positive data after each connected group; ROW = after every row</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>checker.flow</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>LATER</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>admin login only for now</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>res_status.values</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>A,B,C,D</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>CKYC 7.0 values</t>
         </is>
@@ -2433,6 +2486,157 @@
       <formula1>"PASS,FAIL,BLOCKED,NOT RUN,RE-RUN"</formula1>
     </dataValidation>
   </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:V1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Run_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp_IST</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>TC_ID</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Customer_ID</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Persona</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Tab</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Field_Locator_ID</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Value_Before</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Value_Entered</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Value_After</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>Inline_Error</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>Toast_Text</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>Dialog_Text</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>Item_Error_List</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>API_Status</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>Screenshot_Path</t>
+        </is>
+      </c>
+      <c r="U1" s="2" t="inlineStr">
+        <is>
+          <t>Step_Result</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
+        <is>
+          <t>Duration_ms</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:V1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>